<commit_message>
Small changes in analysis code
</commit_message>
<xml_diff>
--- a/tables/ae_per_resource_metrics.xlsx
+++ b/tables/ae_per_resource_metrics.xlsx
@@ -490,17 +490,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.751</t>
+          <t>0.762</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.595</t>
+          <t>0.610</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.664</t>
+          <t>0.677</t>
         </is>
       </c>
     </row>
@@ -518,17 +518,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.711</t>
+          <t>0.725</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.537</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.587</t>
+          <t>0.617</t>
         </is>
       </c>
     </row>
@@ -546,17 +546,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.677</t>
+          <t>0.722</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.412</t>
+          <t>0.510</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.512</t>
+          <t>0.598</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.850</t>
+          <t>0.844</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.845</t>
+          <t>0.804</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.847</t>
+          <t>0.824</t>
         </is>
       </c>
     </row>
@@ -602,17 +602,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.809</t>
+          <t>0.800</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.734</t>
+          <t>0.763</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.770</t>
+          <t>0.781</t>
         </is>
       </c>
     </row>
@@ -630,17 +630,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.686</t>
+          <t>0.650</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.454</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.546</t>
+          <t>0.496</t>
         </is>
       </c>
     </row>
@@ -658,17 +658,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.846</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.957</t>
+          <t>0.870</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.898</t>
+          <t>0.851</t>
         </is>
       </c>
     </row>
@@ -686,17 +686,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.851</t>
+          <t>0.829</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.952</t>
+          <t>0.810</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.899</t>
+          <t>0.819</t>
         </is>
       </c>
     </row>
@@ -714,17 +714,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.818</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.621</t>
+          <t>0.448</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.706</t>
+          <t>0.565</t>
         </is>
       </c>
     </row>
@@ -742,17 +742,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.706</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.511</t>
+          <t>0.638</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.593</t>
+          <t>0.674</t>
         </is>
       </c>
     </row>
@@ -770,17 +770,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.750</t>
+          <t>0.756</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.750</t>
+          <t>0.773</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.750</t>
+          <t>0.764</t>
         </is>
       </c>
     </row>
@@ -826,17 +826,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.734</t>
+          <t>0.718</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.645</t>
+          <t>0.634</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.687</t>
+          <t>0.673</t>
         </is>
       </c>
     </row>
@@ -854,17 +854,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.728</t>
+          <t>0.697</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.608</t>
+          <t>0.510</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.663</t>
+          <t>0.589</t>
         </is>
       </c>
     </row>

</xml_diff>